<commit_message>
daily-agenda: evening round 2026-07-26 (21:04) — 1 done, 5 open, 1 cancelled
Auto-fired via session-bound trigger. שער המלך done; rest roll over.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CFPjvwjh7GCCjswWwAMZQ8
</commit_message>
<xml_diff>
--- a/.claude/skills/daily-agenda/state/activity-log.xlsx
+++ b/.claude/skills/daily-agenda/state/activity-log.xlsx
@@ -499,7 +499,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>יתגלגל למחר; הודעת וואטסאפ מוכנה ביומן</t>
+          <t>יתגלגל למחר</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,11 @@
           <t>לא בוצע</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>סוכם היום; נשאר לקרוא פסק הרש"פ במלואו</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -589,7 +593,11 @@
           <t>לא בוצע</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>סוכם היום</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -617,7 +625,11 @@
           <t>לא בוצע</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>סוכם היום</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -642,7 +654,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>לא בוצע</t>
+          <t>בוצע</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>

</xml_diff>